<commit_message>
final codes and outputs of the WWTP inflow model - constrained and unconstrained
</commit_message>
<xml_diff>
--- a/results/output_of_models.xlsx
+++ b/results/output_of_models.xlsx
@@ -8,24 +8,36 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/mr861_exeter_ac_uk/Documents/Desktop/model_Faf/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="11_F25DC773A252ABDACC10484C319C55345ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08551FF1-A021-4D14-8D50-8B827E36F959}"/>
+  <xr:revisionPtr revIDLastSave="219" documentId="11_F25DC773A252ABDACC10484C319C55345ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD546137-0836-4927-8BD2-3C0B443A6911}"/>
   <bookViews>
-    <workbookView xWindow="9446" yWindow="591" windowWidth="22817" windowHeight="13132" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GPR-WWTP_Inflow" sheetId="1" r:id="rId1"/>
+    <sheet name="GPR-CSO" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="18">
   <si>
     <t xml:space="preserve">model </t>
   </si>
@@ -64,13 +76,28 @@
   </si>
   <si>
     <t>constraints</t>
+  </si>
+  <si>
+    <t>Sparsification</t>
+  </si>
+  <si>
+    <t>SGPR_constraint</t>
+  </si>
+  <si>
+    <t>Inducing points:</t>
+  </si>
+  <si>
+    <t>execution time (s)</t>
+  </si>
+  <si>
+    <t>% improvement of RMSE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -98,6 +125,19 @@
       <name val="Centaur"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Centaur"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Centaur"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -119,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -130,8 +170,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -417,10 +463,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr defaultRowHeight="18.45" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="22.15234375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="18.3828125" style="1" customWidth="1"/>
     <col min="2" max="2" width="15.07421875" style="2" customWidth="1"/>
     <col min="3" max="3" width="16.69140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="17.84375" style="2" customWidth="1"/>
@@ -428,10 +474,14 @@
     <col min="6" max="7" width="15.765625" style="2" customWidth="1"/>
     <col min="8" max="8" width="14.23046875" style="2" customWidth="1"/>
     <col min="9" max="9" width="15" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="9.23046875" style="2"/>
+    <col min="10" max="10" width="17" style="2" customWidth="1"/>
+    <col min="11" max="11" width="19.84375" style="2" customWidth="1"/>
+    <col min="12" max="13" width="19.3046875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="18.4609375" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="9.23046875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -459,8 +509,23 @@
       <c r="I1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="J1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -489,9 +554,20 @@
         <v>2021</v>
       </c>
       <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="K2" s="3">
+        <v>2019</v>
+      </c>
+      <c r="L2" s="2">
+        <v>2021</v>
+      </c>
+      <c r="M2" s="3">
+        <v>2019</v>
+      </c>
+      <c r="N2" s="2">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -507,10 +583,10 @@
       <c r="E3" s="2">
         <v>32.119999999999997</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="2">
         <v>25.654</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="2">
         <v>33.387999999999998</v>
       </c>
       <c r="H3" s="2">
@@ -519,8 +595,20 @@
       <c r="I3" s="2">
         <v>29.975000000000001</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="K3" s="2">
+        <v>25.905000000000001</v>
+      </c>
+      <c r="L3" s="2">
+        <v>31.143000000000001</v>
+      </c>
+      <c r="M3" s="2">
+        <v>25.712</v>
+      </c>
+      <c r="N3" s="2">
+        <v>31.068999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -536,10 +624,10 @@
       <c r="E4" s="2">
         <v>20.096</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="2">
         <v>17.672000000000001</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="2">
         <v>19.23</v>
       </c>
       <c r="H4" s="2">
@@ -548,8 +636,20 @@
       <c r="I4" s="2">
         <v>18.036999999999999</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="K4" s="2">
+        <v>17.88</v>
+      </c>
+      <c r="L4" s="2">
+        <v>17.771999999999998</v>
+      </c>
+      <c r="M4" s="2">
+        <v>17.704999999999998</v>
+      </c>
+      <c r="N4" s="2">
+        <v>23.721</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -565,10 +665,10 @@
       <c r="E5" s="2">
         <v>88.15</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <v>93.346999999999994</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="2">
         <v>88.15</v>
       </c>
       <c r="H5" s="2">
@@ -577,8 +677,20 @@
       <c r="I5" s="2">
         <v>87.94</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="K5" s="2">
+        <v>94.59</v>
+      </c>
+      <c r="L5" s="2">
+        <v>87.11</v>
+      </c>
+      <c r="M5" s="2">
+        <v>96.67</v>
+      </c>
+      <c r="N5" s="2">
+        <v>94.8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
@@ -594,10 +706,10 @@
       <c r="E6" s="2">
         <v>6.2887000000000004</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="2">
         <v>6.6723999999999997</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="2">
         <v>6.2664</v>
       </c>
       <c r="H6" s="2">
@@ -606,12 +718,20 @@
       <c r="I6" s="2">
         <v>6.1558999999999999</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="K6" s="2">
+        <v>6.78</v>
+      </c>
+      <c r="L6" s="2">
+        <v>6.2442000000000002</v>
+      </c>
+      <c r="M6" s="2">
+        <v>7.2089999999999996</v>
+      </c>
+      <c r="N6" s="2">
+        <v>7.2149999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -627,10 +747,10 @@
       <c r="E8" s="2">
         <v>120</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="2">
         <v>120</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="2">
         <v>120</v>
       </c>
       <c r="H8" s="2">
@@ -639,8 +759,49 @@
       <c r="I8" s="2">
         <v>120</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="J8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="3">
+        <v>100</v>
+      </c>
+      <c r="L8" s="3">
+        <v>100</v>
+      </c>
+      <c r="M8" s="3">
+        <v>500</v>
+      </c>
+      <c r="N8" s="3">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="2">
+        <v>220</v>
+      </c>
+      <c r="I9" s="2">
+        <v>246</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K9" s="2">
+        <v>18</v>
+      </c>
+      <c r="L9" s="2">
+        <v>22</v>
+      </c>
+      <c r="M9" s="2">
+        <v>268</v>
+      </c>
+      <c r="N9" s="2">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="F10" s="2" t="s">
         <v>10</v>
       </c>
@@ -652,6 +813,270 @@
       </c>
       <c r="I10" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="36.9" x14ac:dyDescent="0.4">
+      <c r="A12" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="2">
+        <f>-100*(B3 - $B3)/$B3</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="2">
+        <f>-100*(C3 - $C3)/$C3</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="2">
+        <f>-100*(D3 - $B3)/$B3</f>
+        <v>24.741246100469404</v>
+      </c>
+      <c r="E12" s="2">
+        <f>-100*(E3 - $C3)/$C3</f>
+        <v>23.064025485640386</v>
+      </c>
+      <c r="F12" s="2">
+        <f>-100*(F3 - $B3)/$B3</f>
+        <v>25.204816466952391</v>
+      </c>
+      <c r="G12" s="2">
+        <f>-100*(G3 - $C3)/$C3</f>
+        <v>20.026826989868027</v>
+      </c>
+      <c r="H12" s="2">
+        <f>-100*(H3 - $B3)/$B3</f>
+        <v>25.455552640018652</v>
+      </c>
+      <c r="I12" s="2">
+        <f>-100*(I3 - $C3)/$C3</f>
+        <v>28.201873098756856</v>
+      </c>
+      <c r="K12" s="2">
+        <f>-100*(K3 - $H3)/$H3</f>
+        <v>-1.3180538172715883</v>
+      </c>
+      <c r="L12" s="2">
+        <f>-100*(L3 - $I3)/$I3</f>
+        <v>-3.8965804837364444</v>
+      </c>
+      <c r="M12" s="2">
+        <f>-100*(M3 - $H3)/$H3</f>
+        <v>-0.56320400500625134</v>
+      </c>
+      <c r="N12" s="2">
+        <f>-100*(N3 - $I3)/$I3</f>
+        <v>-3.6497080900750545</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="K13" s="2">
+        <f>-100*(K4 - $H4)/$H4</f>
+        <v>-1.4180374361883155</v>
+      </c>
+      <c r="L13" s="2">
+        <f>-100*(L4 - $I4)/$I4</f>
+        <v>1.4692021954870575</v>
+      </c>
+      <c r="M13" s="2">
+        <f>-100*(M4 - $H4)/$H4</f>
+        <v>-0.42541123085649063</v>
+      </c>
+      <c r="N13" s="2">
+        <f>-100*(N4 - $I4)/$I4</f>
+        <v>-31.513001053390258</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="K14" s="2">
+        <f t="shared" ref="K14:K15" si="0">-100*(K5 - $H5)/$H5</f>
+        <v>-1.7862907564833708</v>
+      </c>
+      <c r="L14" s="2">
+        <f t="shared" ref="L14:L15" si="1">-100*(L5 - $I5)/$I5</f>
+        <v>0.94382533545599079</v>
+      </c>
+      <c r="M14" s="2">
+        <f t="shared" ref="M14:M15" si="2">-100*(M5 - $H5)/$H5</f>
+        <v>-4.0245345959324164</v>
+      </c>
+      <c r="N14" s="2">
+        <f t="shared" ref="N14:N15" si="3">-100*(N5 - $I5)/$I5</f>
+        <v>-7.8007732544916992</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="K15" s="2">
+        <f t="shared" si="0"/>
+        <v>-2.3937174356263697</v>
+      </c>
+      <c r="L15" s="2">
+        <f t="shared" si="1"/>
+        <v>-1.4343962702448101</v>
+      </c>
+      <c r="M15" s="2">
+        <f t="shared" si="2"/>
+        <v>-8.8726119459336914</v>
+      </c>
+      <c r="N15" s="2">
+        <f t="shared" si="3"/>
+        <v>-17.204632953751684</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E923AD0-BD79-4D6A-B13C-DB02488FEFDA}">
+  <dimension ref="A1:N12"/>
+  <sheetFormatPr defaultRowHeight="18.45" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="18.3828125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.07421875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="16.69140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.84375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="16.61328125" style="2" customWidth="1"/>
+    <col min="6" max="7" width="15.765625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="14.23046875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="15" style="2" customWidth="1"/>
+    <col min="10" max="10" width="17" style="2" customWidth="1"/>
+    <col min="11" max="11" width="19.84375" style="2" customWidth="1"/>
+    <col min="12" max="13" width="19.3046875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="18.4609375" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="9.23046875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2019</v>
+      </c>
+      <c r="C2" s="3">
+        <v>2021</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2019</v>
+      </c>
+      <c r="E2" s="3">
+        <v>2021</v>
+      </c>
+      <c r="F2" s="3">
+        <v>2019</v>
+      </c>
+      <c r="G2" s="3">
+        <v>2021</v>
+      </c>
+      <c r="H2" s="3">
+        <v>2019</v>
+      </c>
+      <c r="I2" s="3">
+        <v>2021</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3">
+        <v>2019</v>
+      </c>
+      <c r="L2" s="2">
+        <v>2021</v>
+      </c>
+      <c r="M2" s="3">
+        <v>2019</v>
+      </c>
+      <c r="N2" s="2">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A6" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="36.9" x14ac:dyDescent="0.4">
+      <c r="A12" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>